<commit_message>
fix: make review frame-accurate and correct escape, strategy, and speed
Manual review now steps source frames and edits investigations. Escape inference ignores future target visits, strategy reasoning uses chronological transition counts, and mean speed is time-weighted.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/examples/outputs/barnes-maze-sample-results.xlsx
+++ b/examples/outputs/barnes-maze-sample-results.xlsx
@@ -194,7 +194,7 @@
     <t>analyzed_at</t>
   </si>
   <si>
-    <t>2026-08-31T20:30:48.405Z</t>
+    <t>2026-08-31T21:53:33.193Z</t>
   </si>
   <si>
     <t>sampling</t>
@@ -828,7 +828,7 @@
         <v>1253.7852830989489</v>
       </c>
       <c r="L2">
-        <v>6.980987099660074</v>
+        <v>6.980987099660072</v>
       </c>
       <c r="M2">
         <v>82.33333333333333</v>
@@ -872,7 +872,7 @@
         <v>217.57802025036344</v>
       </c>
       <c r="L3">
-        <v>4.405959316029171</v>
+        <v>4.4059593160291755</v>
       </c>
       <c r="M3">
         <v>18.685333333333332</v>
@@ -916,7 +916,7 @@
         <v>105.52461561712477</v>
       </c>
       <c r="L4">
-        <v>4.198592133307352</v>
+        <v>4.1985921333073515</v>
       </c>
       <c r="M4">
         <v>25.133333333333333</v>

</xml_diff>